<commit_message>
Updated FRA model - 2025-09-13 09:14
</commit_message>
<xml_diff>
--- a/VerveStacks_FRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_FRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_FRA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2643E9D-F298-4355-BC63-3D1086B587D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C680789A-9E77-4023-9E06-B6EF784818CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -994,18 +994,18 @@
     <t>onshore wind resource -- CF class won-FRA_59 -- cost class 1</t>
   </si>
   <si>
+    <t>e_won-FRA_59_c4</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_59 -- cost class 4</t>
+  </si>
+  <si>
     <t>e_won-FRA_59_c3</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_59 -- cost class 3</t>
   </si>
   <si>
-    <t>e_won-FRA_59_c4</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_59 -- cost class 4</t>
-  </si>
-  <si>
     <t>e_won-FRA_58_c1</t>
   </si>
   <si>
@@ -1072,16 +1072,22 @@
     <t>onshore wind resource -- CF class won-FRA_56 -- cost class 2</t>
   </si>
   <si>
+    <t>e_won-FRA_55_c1</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_55 -- cost class 1</t>
+  </si>
+  <si>
     <t>e_won-FRA_55_c2</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_55 -- cost class 2</t>
   </si>
   <si>
-    <t>e_won-FRA_55_c1</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_55 -- cost class 1</t>
+    <t>e_won-FRA_54_c3</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_54 -- cost class 3</t>
   </si>
   <si>
     <t>e_won-FRA_54_c4</t>
@@ -1090,10 +1096,10 @@
     <t>onshore wind resource -- CF class won-FRA_54 -- cost class 4</t>
   </si>
   <si>
-    <t>e_won-FRA_54_c3</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_54 -- cost class 3</t>
+    <t>e_won-FRA_54_c1</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_54 -- cost class 1</t>
   </si>
   <si>
     <t>e_won-FRA_54_c2</t>
@@ -1102,30 +1108,24 @@
     <t>onshore wind resource -- CF class won-FRA_54 -- cost class 2</t>
   </si>
   <si>
-    <t>e_won-FRA_54_c1</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_54 -- cost class 1</t>
-  </si>
-  <si>
     <t>e_won-FRA_53_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_53 -- cost class 1</t>
   </si>
   <si>
+    <t>e_won-FRA_53_c4</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_53 -- cost class 4</t>
+  </si>
+  <si>
     <t>e_won-FRA_53_c5</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_53 -- cost class 5</t>
   </si>
   <si>
-    <t>e_won-FRA_53_c4</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_53 -- cost class 4</t>
-  </si>
-  <si>
     <t>e_won-FRA_53_c3</t>
   </si>
   <si>
@@ -1138,16 +1138,22 @@
     <t>onshore wind resource -- CF class won-FRA_53 -- cost class 2</t>
   </si>
   <si>
+    <t>e_won-FRA_50_c4</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_50 -- cost class 4</t>
+  </si>
+  <si>
     <t>e_won-FRA_50_c3</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_50 -- cost class 3</t>
   </si>
   <si>
-    <t>e_won-FRA_50_c4</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_50 -- cost class 4</t>
+    <t>e_won-FRA_50_c2</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_50 -- cost class 2</t>
   </si>
   <si>
     <t>e_won-FRA_50_c1</t>
@@ -1156,12 +1162,6 @@
     <t>onshore wind resource -- CF class won-FRA_50 -- cost class 1</t>
   </si>
   <si>
-    <t>e_won-FRA_50_c2</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_50 -- cost class 2</t>
-  </si>
-  <si>
     <t>e_won-FRA_49_c3</t>
   </si>
   <si>
@@ -1174,36 +1174,36 @@
     <t>onshore wind resource -- CF class won-FRA_49 -- cost class 2</t>
   </si>
   <si>
+    <t>e_won-FRA_49_c4</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_49 -- cost class 4</t>
+  </si>
+  <si>
     <t>e_won-FRA_49_c5</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_49 -- cost class 5</t>
   </si>
   <si>
-    <t>e_won-FRA_49_c4</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_49 -- cost class 4</t>
-  </si>
-  <si>
     <t>e_won-FRA_49_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_49 -- cost class 1</t>
   </si>
   <si>
+    <t>e_won-FRA_48_c1</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_48 -- cost class 1</t>
+  </si>
+  <si>
     <t>e_won-FRA_48_c2</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_48 -- cost class 2</t>
   </si>
   <si>
-    <t>e_won-FRA_48_c1</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_48 -- cost class 1</t>
-  </si>
-  <si>
     <t>e_won-FRA_48_c4</t>
   </si>
   <si>
@@ -1282,16 +1282,22 @@
     <t>onshore wind resource -- CF class won-FRA_45 -- cost class 1</t>
   </si>
   <si>
+    <t>e_won-FRA_45_c3</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_45 -- cost class 3</t>
+  </si>
+  <si>
     <t>e_won-FRA_45_c4</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_45 -- cost class 4</t>
   </si>
   <si>
-    <t>e_won-FRA_45_c3</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_45 -- cost class 3</t>
+    <t>e_won-FRA_43_c4</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_43 -- cost class 4</t>
   </si>
   <si>
     <t>e_won-FRA_43_c3</t>
@@ -1300,12 +1306,6 @@
     <t>onshore wind resource -- CF class won-FRA_43 -- cost class 3</t>
   </si>
   <si>
-    <t>e_won-FRA_43_c4</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_43 -- cost class 4</t>
-  </si>
-  <si>
     <t>e_won-FRA_43_c2</t>
   </si>
   <si>
@@ -1336,18 +1336,18 @@
     <t>onshore wind resource -- CF class won-FRA_41 -- cost class 1</t>
   </si>
   <si>
+    <t>e_won-FRA_41_c5</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_41 -- cost class 5</t>
+  </si>
+  <si>
     <t>e_won-FRA_41_c4</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_41 -- cost class 4</t>
   </si>
   <si>
-    <t>e_won-FRA_41_c5</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_41 -- cost class 5</t>
-  </si>
-  <si>
     <t>e_won-FRA_41_c3</t>
   </si>
   <si>
@@ -1360,34 +1360,40 @@
     <t>onshore wind resource -- CF class won-FRA_41 -- cost class 2</t>
   </si>
   <si>
+    <t>e_won-FRA_40_c3</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_40 -- cost class 3</t>
+  </si>
+  <si>
     <t>e_won-FRA_40_c2</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_40 -- cost class 2</t>
   </si>
   <si>
-    <t>e_won-FRA_40_c3</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_40 -- cost class 3</t>
-  </si>
-  <si>
     <t>e_won-FRA_40_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_40 -- cost class 1</t>
   </si>
   <si>
+    <t>e_won-FRA_40_c4</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_40 -- cost class 4</t>
+  </si>
+  <si>
     <t>e_won-FRA_40_c5</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_40 -- cost class 5</t>
   </si>
   <si>
-    <t>e_won-FRA_40_c4</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_40 -- cost class 4</t>
+    <t>e_won-FRA_39_c4</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_39 -- cost class 4</t>
   </si>
   <si>
     <t>e_won-FRA_39_c3</t>
@@ -1396,12 +1402,6 @@
     <t>onshore wind resource -- CF class won-FRA_39 -- cost class 3</t>
   </si>
   <si>
-    <t>e_won-FRA_39_c4</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_39 -- cost class 4</t>
-  </si>
-  <si>
     <t>e_won-FRA_39_c1</t>
   </si>
   <si>
@@ -2200,18 +2200,18 @@
     <t>onshore wind resource -- CF class won-FRA_10 -- cost class 1</t>
   </si>
   <si>
+    <t>e_won-FRA_10_c3</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_10 -- cost class 3</t>
+  </si>
+  <si>
     <t>e_won-FRA_10_c4</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_10 -- cost class 4</t>
   </si>
   <si>
-    <t>e_won-FRA_10_c3</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_10 -- cost class 3</t>
-  </si>
-  <si>
     <t>e_won-FRA_9_c2</t>
   </si>
   <si>
@@ -2224,16 +2224,22 @@
     <t>onshore wind resource -- CF class won-FRA_9 -- cost class 1</t>
   </si>
   <si>
+    <t>e_won-FRA_9_c4</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_9 -- cost class 4</t>
+  </si>
+  <si>
     <t>e_won-FRA_9_c3</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_9 -- cost class 3</t>
   </si>
   <si>
-    <t>e_won-FRA_9_c4</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_9 -- cost class 4</t>
+    <t>e_won-FRA_8_c5</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_8 -- cost class 5</t>
   </si>
   <si>
     <t>e_won-FRA_8_c4</t>
@@ -2242,12 +2248,6 @@
     <t>onshore wind resource -- CF class won-FRA_8 -- cost class 4</t>
   </si>
   <si>
-    <t>e_won-FRA_8_c5</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_8 -- cost class 5</t>
-  </si>
-  <si>
     <t>e_won-FRA_8_c3</t>
   </si>
   <si>
@@ -2326,16 +2326,16 @@
     <t>onshore wind resource -- CF class won-FRA_5 -- cost class 3</t>
   </si>
   <si>
+    <t>e_won-FRA_4_c3</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_4 -- cost class 3</t>
+  </si>
+  <si>
     <t>e_won-FRA_4_c2</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_4 -- cost class 2</t>
-  </si>
-  <si>
-    <t>e_won-FRA_4_c3</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_4 -- cost class 3</t>
   </si>
   <si>
     <t>e_won-FRA_4_c1</t>
@@ -8016,7 +8016,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{326D7A16-709E-4247-9ABB-9399DEB63957}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7F57F98-29A8-46AB-B6CA-C2871539405A}">
   <dimension ref="B9:N55"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9782,7 +9782,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D1F468F-5896-47CE-AE09-5BCAD7A1A6CC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{472EE37A-E776-4035-9580-A4DE53FC1CEC}">
   <dimension ref="B9:AB253"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10205,7 +10205,7 @@
         <v>0.5869329005007935</v>
       </c>
       <c r="N15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P15" t="s">
         <v>182</v>
@@ -10279,7 +10279,7 @@
         <v>0.5869329005007935</v>
       </c>
       <c r="N16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P16" t="s">
         <v>182</v>
@@ -11167,7 +11167,7 @@
         <v>0.5481425465611397</v>
       </c>
       <c r="N28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P28" t="s">
         <v>182</v>
@@ -11241,7 +11241,7 @@
         <v>0.5481425465611397</v>
       </c>
       <c r="N29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P29" t="s">
         <v>182</v>
@@ -11315,7 +11315,7 @@
         <v>0.54203381698000042</v>
       </c>
       <c r="N30">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P30" t="s">
         <v>182</v>
@@ -11389,7 +11389,7 @@
         <v>0.54203381698000042</v>
       </c>
       <c r="N31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P31" t="s">
         <v>182</v>
@@ -11463,7 +11463,7 @@
         <v>0.53797007154491827</v>
       </c>
       <c r="N32">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P32" t="s">
         <v>182</v>
@@ -11537,7 +11537,7 @@
         <v>0.53797007154491827</v>
       </c>
       <c r="N33">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P33" t="s">
         <v>182</v>
@@ -11685,7 +11685,7 @@
         <v>0.53220597567372174</v>
       </c>
       <c r="N35">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P35" t="s">
         <v>182</v>
@@ -11759,7 +11759,7 @@
         <v>0.53220597567372174</v>
       </c>
       <c r="N36">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P36" t="s">
         <v>182</v>
@@ -11981,7 +11981,7 @@
         <v>0.50220459612144741</v>
       </c>
       <c r="N39">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P39" t="s">
         <v>182</v>
@@ -12055,7 +12055,7 @@
         <v>0.50220459612144741</v>
       </c>
       <c r="N40">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P40" t="s">
         <v>182</v>
@@ -12129,7 +12129,7 @@
         <v>0.49522886431330682</v>
       </c>
       <c r="N41">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P41" t="s">
         <v>182</v>
@@ -12203,7 +12203,7 @@
         <v>0.49522886431330682</v>
       </c>
       <c r="N42">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P42" t="s">
         <v>182</v>
@@ -12425,7 +12425,7 @@
         <v>0.48997678015376445</v>
       </c>
       <c r="N45">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P45" t="s">
         <v>182</v>
@@ -12499,7 +12499,7 @@
         <v>0.48997678015376445</v>
       </c>
       <c r="N46">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P46" t="s">
         <v>182</v>
@@ -12647,7 +12647,7 @@
         <v>0.48274206530326413</v>
       </c>
       <c r="N48">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P48" t="s">
         <v>182</v>
@@ -12721,7 +12721,7 @@
         <v>0.48274206530326413</v>
       </c>
       <c r="N49">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P49" t="s">
         <v>182</v>
@@ -13757,7 +13757,7 @@
         <v>0.44927182040159591</v>
       </c>
       <c r="N63">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P63" t="s">
         <v>182</v>
@@ -13831,7 +13831,7 @@
         <v>0.44927182040159591</v>
       </c>
       <c r="N64">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P64" t="s">
         <v>182</v>
@@ -13905,7 +13905,7 @@
         <v>0.4311669102324972</v>
       </c>
       <c r="N65">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P65" t="s">
         <v>182</v>
@@ -13979,7 +13979,7 @@
         <v>0.4311669102324972</v>
       </c>
       <c r="N66">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P66" t="s">
         <v>182</v>
@@ -14423,7 +14423,7 @@
         <v>0.41247392735747213</v>
       </c>
       <c r="N72">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P72" t="s">
         <v>182</v>
@@ -14497,7 +14497,7 @@
         <v>0.41247392735747213</v>
       </c>
       <c r="N73">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P73" t="s">
         <v>182</v>
@@ -14719,7 +14719,7 @@
         <v>0.40413001707392909</v>
       </c>
       <c r="N76">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P76" t="s">
         <v>182</v>
@@ -14793,7 +14793,7 @@
         <v>0.40413001707392909</v>
       </c>
       <c r="N77">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P77" t="s">
         <v>182</v>
@@ -14941,7 +14941,7 @@
         <v>0.3980373835402759</v>
       </c>
       <c r="N79">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P79" t="s">
         <v>182</v>
@@ -15015,7 +15015,7 @@
         <v>0.3980373835402759</v>
       </c>
       <c r="N80">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P80" t="s">
         <v>182</v>
@@ -15089,7 +15089,7 @@
         <v>0.39372775589879089</v>
       </c>
       <c r="N81">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P81" t="s">
         <v>182</v>
@@ -15163,7 +15163,7 @@
         <v>0.39372775589879089</v>
       </c>
       <c r="N82">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P82" t="s">
         <v>182</v>
@@ -21587,7 +21587,7 @@
         <v>9.6601232604683201E-2</v>
       </c>
       <c r="N216">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="217" spans="2:14">
@@ -21625,7 +21625,7 @@
         <v>9.6601232604683201E-2</v>
       </c>
       <c r="N217">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="218" spans="2:14">
@@ -21739,7 +21739,7 @@
         <v>9.0232523202525394E-2</v>
       </c>
       <c r="N220">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="221" spans="2:14">
@@ -21777,7 +21777,7 @@
         <v>9.0232523202525394E-2</v>
       </c>
       <c r="N221">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="222" spans="2:14">
@@ -21815,7 +21815,7 @@
         <v>8.3146820266911795E-2</v>
       </c>
       <c r="N222">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="223" spans="2:14">
@@ -21853,7 +21853,7 @@
         <v>8.3146820266911795E-2</v>
       </c>
       <c r="N223">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="224" spans="2:14">
@@ -22385,7 +22385,7 @@
         <v>4.4893033534251302E-2</v>
       </c>
       <c r="N237">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="238" spans="2:14">
@@ -22423,7 +22423,7 @@
         <v>4.4893033534251302E-2</v>
       </c>
       <c r="N238">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="239" spans="2:14">
@@ -23002,7 +23002,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08BE8D5A-4C59-43A0-8CC4-9277F7B854B7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE099407-1872-420B-998F-B75BBFE06647}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated FRA model - 2025-09-13 09:55
</commit_message>
<xml_diff>
--- a/VerveStacks_FRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_FRA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_FRA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C680789A-9E77-4023-9E06-B6EF784818CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{72F61B30-8E33-455E-8BAB-10B3C379B67F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -970,18 +970,18 @@
     <t>elc_spv-FRA</t>
   </si>
   <si>
+    <t>e_won-FRA_60_c2</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_60 -- cost class 2</t>
+  </si>
+  <si>
     <t>e_won-FRA_60_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_60 -- cost class 1</t>
   </si>
   <si>
-    <t>e_won-FRA_60_c2</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_60 -- cost class 2</t>
-  </si>
-  <si>
     <t>e_won-FRA_59_c2</t>
   </si>
   <si>
@@ -1042,34 +1042,40 @@
     <t>onshore wind resource -- CF class won-FRA_57 -- cost class 2</t>
   </si>
   <si>
+    <t>e_won-FRA_57_c4</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_57 -- cost class 4</t>
+  </si>
+  <si>
     <t>e_won-FRA_57_c5</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_57 -- cost class 5</t>
   </si>
   <si>
-    <t>e_won-FRA_57_c4</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_57 -- cost class 4</t>
-  </si>
-  <si>
     <t>e_won-FRA_57_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_57 -- cost class 1</t>
   </si>
   <si>
+    <t>e_won-FRA_56_c2</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_56 -- cost class 2</t>
+  </si>
+  <si>
     <t>e_won-FRA_56_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_56 -- cost class 1</t>
   </si>
   <si>
-    <t>e_won-FRA_56_c2</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_56 -- cost class 2</t>
+    <t>e_won-FRA_55_c2</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_55 -- cost class 2</t>
   </si>
   <si>
     <t>e_won-FRA_55_c1</t>
@@ -1078,12 +1084,6 @@
     <t>onshore wind resource -- CF class won-FRA_55 -- cost class 1</t>
   </si>
   <si>
-    <t>e_won-FRA_55_c2</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_55 -- cost class 2</t>
-  </si>
-  <si>
     <t>e_won-FRA_54_c3</t>
   </si>
   <si>
@@ -1096,36 +1096,36 @@
     <t>onshore wind resource -- CF class won-FRA_54 -- cost class 4</t>
   </si>
   <si>
+    <t>e_won-FRA_54_c2</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_54 -- cost class 2</t>
+  </si>
+  <si>
     <t>e_won-FRA_54_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_54 -- cost class 1</t>
   </si>
   <si>
-    <t>e_won-FRA_54_c2</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_54 -- cost class 2</t>
-  </si>
-  <si>
     <t>e_won-FRA_53_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_53 -- cost class 1</t>
   </si>
   <si>
+    <t>e_won-FRA_53_c5</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_53 -- cost class 5</t>
+  </si>
+  <si>
     <t>e_won-FRA_53_c4</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_53 -- cost class 4</t>
   </si>
   <si>
-    <t>e_won-FRA_53_c5</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_53 -- cost class 5</t>
-  </si>
-  <si>
     <t>e_won-FRA_53_c3</t>
   </si>
   <si>
@@ -1138,16 +1138,22 @@
     <t>onshore wind resource -- CF class won-FRA_53 -- cost class 2</t>
   </si>
   <si>
+    <t>e_won-FRA_50_c3</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_50 -- cost class 3</t>
+  </si>
+  <si>
     <t>e_won-FRA_50_c4</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_50 -- cost class 4</t>
   </si>
   <si>
-    <t>e_won-FRA_50_c3</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_50 -- cost class 3</t>
+    <t>e_won-FRA_50_c1</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_50 -- cost class 1</t>
   </si>
   <si>
     <t>e_won-FRA_50_c2</t>
@@ -1156,12 +1162,6 @@
     <t>onshore wind resource -- CF class won-FRA_50 -- cost class 2</t>
   </si>
   <si>
-    <t>e_won-FRA_50_c1</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_50 -- cost class 1</t>
-  </si>
-  <si>
     <t>e_won-FRA_49_c3</t>
   </si>
   <si>
@@ -1174,34 +1174,40 @@
     <t>onshore wind resource -- CF class won-FRA_49 -- cost class 2</t>
   </si>
   <si>
+    <t>e_won-FRA_49_c5</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_49 -- cost class 5</t>
+  </si>
+  <si>
     <t>e_won-FRA_49_c4</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_49 -- cost class 4</t>
   </si>
   <si>
-    <t>e_won-FRA_49_c5</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_49 -- cost class 5</t>
-  </si>
-  <si>
     <t>e_won-FRA_49_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_49 -- cost class 1</t>
   </si>
   <si>
+    <t>e_won-FRA_48_c2</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_48 -- cost class 2</t>
+  </si>
+  <si>
     <t>e_won-FRA_48_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_48 -- cost class 1</t>
   </si>
   <si>
-    <t>e_won-FRA_48_c2</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_48 -- cost class 2</t>
+    <t>e_won-FRA_48_c3</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_48 -- cost class 3</t>
   </si>
   <si>
     <t>e_won-FRA_48_c4</t>
@@ -1210,12 +1216,6 @@
     <t>onshore wind resource -- CF class won-FRA_48 -- cost class 4</t>
   </si>
   <si>
-    <t>e_won-FRA_48_c3</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_48 -- cost class 3</t>
-  </si>
-  <si>
     <t>e_won-FRA_47_c4</t>
   </si>
   <si>
@@ -1246,16 +1246,22 @@
     <t>onshore wind resource -- CF class won-FRA_47 -- cost class 5</t>
   </si>
   <si>
+    <t>e_won-FRA_46_c4</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_46 -- cost class 4</t>
+  </si>
+  <si>
     <t>e_won-FRA_46_c3</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_46 -- cost class 3</t>
   </si>
   <si>
-    <t>e_won-FRA_46_c4</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_46 -- cost class 4</t>
+    <t>e_won-FRA_46_c2</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_46 -- cost class 2</t>
   </si>
   <si>
     <t>e_won-FRA_46_c1</t>
@@ -1264,10 +1270,10 @@
     <t>onshore wind resource -- CF class won-FRA_46 -- cost class 1</t>
   </si>
   <si>
-    <t>e_won-FRA_46_c2</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_46 -- cost class 2</t>
+    <t>e_won-FRA_45_c1</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_45 -- cost class 1</t>
   </si>
   <si>
     <t>e_won-FRA_45_c2</t>
@@ -1276,10 +1282,10 @@
     <t>onshore wind resource -- CF class won-FRA_45 -- cost class 2</t>
   </si>
   <si>
-    <t>e_won-FRA_45_c1</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_45 -- cost class 1</t>
+    <t>e_won-FRA_45_c4</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_45 -- cost class 4</t>
   </si>
   <si>
     <t>e_won-FRA_45_c3</t>
@@ -1288,10 +1294,10 @@
     <t>onshore wind resource -- CF class won-FRA_45 -- cost class 3</t>
   </si>
   <si>
-    <t>e_won-FRA_45_c4</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_45 -- cost class 4</t>
+    <t>e_won-FRA_43_c3</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_43 -- cost class 3</t>
   </si>
   <si>
     <t>e_won-FRA_43_c4</t>
@@ -1300,10 +1306,10 @@
     <t>onshore wind resource -- CF class won-FRA_43 -- cost class 4</t>
   </si>
   <si>
-    <t>e_won-FRA_43_c3</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_43 -- cost class 3</t>
+    <t>e_won-FRA_43_c1</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_43 -- cost class 1</t>
   </si>
   <si>
     <t>e_won-FRA_43_c2</t>
@@ -1312,10 +1318,10 @@
     <t>onshore wind resource -- CF class won-FRA_43 -- cost class 2</t>
   </si>
   <si>
-    <t>e_won-FRA_43_c1</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_43 -- cost class 1</t>
+    <t>e_won-FRA_42_c1</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_42 -- cost class 1</t>
   </si>
   <si>
     <t>e_won-FRA_42_c2</t>
@@ -1324,30 +1330,24 @@
     <t>onshore wind resource -- CF class won-FRA_42 -- cost class 2</t>
   </si>
   <si>
-    <t>e_won-FRA_42_c1</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_42 -- cost class 1</t>
-  </si>
-  <si>
     <t>e_won-FRA_41_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_41 -- cost class 1</t>
   </si>
   <si>
+    <t>e_won-FRA_41_c4</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_41 -- cost class 4</t>
+  </si>
+  <si>
     <t>e_won-FRA_41_c5</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_41 -- cost class 5</t>
   </si>
   <si>
-    <t>e_won-FRA_41_c4</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_41 -- cost class 4</t>
-  </si>
-  <si>
     <t>e_won-FRA_41_c3</t>
   </si>
   <si>
@@ -1360,36 +1360,36 @@
     <t>onshore wind resource -- CF class won-FRA_41 -- cost class 2</t>
   </si>
   <si>
+    <t>e_won-FRA_40_c2</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_40 -- cost class 2</t>
+  </si>
+  <si>
     <t>e_won-FRA_40_c3</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_40 -- cost class 3</t>
   </si>
   <si>
-    <t>e_won-FRA_40_c2</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_40 -- cost class 2</t>
-  </si>
-  <si>
     <t>e_won-FRA_40_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_40 -- cost class 1</t>
   </si>
   <si>
+    <t>e_won-FRA_40_c5</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_40 -- cost class 5</t>
+  </si>
+  <si>
     <t>e_won-FRA_40_c4</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_40 -- cost class 4</t>
   </si>
   <si>
-    <t>e_won-FRA_40_c5</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_40 -- cost class 5</t>
-  </si>
-  <si>
     <t>e_won-FRA_39_c4</t>
   </si>
   <si>
@@ -1402,18 +1402,18 @@
     <t>onshore wind resource -- CF class won-FRA_39 -- cost class 3</t>
   </si>
   <si>
+    <t>e_won-FRA_39_c2</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_39 -- cost class 2</t>
+  </si>
+  <si>
     <t>e_won-FRA_39_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_39 -- cost class 1</t>
   </si>
   <si>
-    <t>e_won-FRA_39_c2</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_39 -- cost class 2</t>
-  </si>
-  <si>
     <t>e_won-FRA_38_c5</t>
   </si>
   <si>
@@ -2074,36 +2074,36 @@
     <t>onshore wind resource -- CF class won-FRA_17 -- cost class 4</t>
   </si>
   <si>
+    <t>e_won-FRA_15_c1</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_15 -- cost class 1</t>
+  </si>
+  <si>
     <t>e_won-FRA_15_c2</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_15 -- cost class 2</t>
   </si>
   <si>
-    <t>e_won-FRA_15_c1</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_15 -- cost class 1</t>
-  </si>
-  <si>
     <t>e_won-FRA_14_c3</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_14 -- cost class 3</t>
   </si>
   <si>
+    <t>e_won-FRA_14_c4</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_14 -- cost class 4</t>
+  </si>
+  <si>
     <t>e_won-FRA_14_c5</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_14 -- cost class 5</t>
   </si>
   <si>
-    <t>e_won-FRA_14_c4</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_14 -- cost class 4</t>
-  </si>
-  <si>
     <t>e_won-FRA_14_c1</t>
   </si>
   <si>
@@ -2116,18 +2116,18 @@
     <t>onshore wind resource -- CF class won-FRA_14 -- cost class 2</t>
   </si>
   <si>
+    <t>e_won-FRA_13_c2</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_13 -- cost class 2</t>
+  </si>
+  <si>
     <t>e_won-FRA_13_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_13 -- cost class 1</t>
   </si>
   <si>
-    <t>e_won-FRA_13_c2</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_13 -- cost class 2</t>
-  </si>
-  <si>
     <t>e_won-FRA_12_c3</t>
   </si>
   <si>
@@ -2158,18 +2158,18 @@
     <t>onshore wind resource -- CF class won-FRA_12 -- cost class 4</t>
   </si>
   <si>
+    <t>e_won-FRA_11_c2</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_11 -- cost class 2</t>
+  </si>
+  <si>
     <t>e_won-FRA_11_c3</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_11 -- cost class 3</t>
   </si>
   <si>
-    <t>e_won-FRA_11_c2</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_11 -- cost class 2</t>
-  </si>
-  <si>
     <t>e_won-FRA_11_c5</t>
   </si>
   <si>
@@ -2188,16 +2188,22 @@
     <t>onshore wind resource -- CF class won-FRA_11 -- cost class 1</t>
   </si>
   <si>
+    <t>e_won-FRA_10_c1</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_10 -- cost class 1</t>
+  </si>
+  <si>
     <t>e_won-FRA_10_c2</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_10 -- cost class 2</t>
   </si>
   <si>
-    <t>e_won-FRA_10_c1</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_10 -- cost class 1</t>
+    <t>e_won-FRA_10_c4</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_10 -- cost class 4</t>
   </si>
   <si>
     <t>e_won-FRA_10_c3</t>
@@ -2206,12 +2212,6 @@
     <t>onshore wind resource -- CF class won-FRA_10 -- cost class 3</t>
   </si>
   <si>
-    <t>e_won-FRA_10_c4</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_10 -- cost class 4</t>
-  </si>
-  <si>
     <t>e_won-FRA_9_c2</t>
   </si>
   <si>
@@ -2236,18 +2236,18 @@
     <t>onshore wind resource -- CF class won-FRA_9 -- cost class 3</t>
   </si>
   <si>
+    <t>e_won-FRA_8_c4</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_8 -- cost class 4</t>
+  </si>
+  <si>
     <t>e_won-FRA_8_c5</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_8 -- cost class 5</t>
   </si>
   <si>
-    <t>e_won-FRA_8_c4</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_8 -- cost class 4</t>
-  </si>
-  <si>
     <t>e_won-FRA_8_c3</t>
   </si>
   <si>
@@ -2326,34 +2326,40 @@
     <t>onshore wind resource -- CF class won-FRA_5 -- cost class 3</t>
   </si>
   <si>
+    <t>e_won-FRA_4_c2</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_4 -- cost class 2</t>
+  </si>
+  <si>
     <t>e_won-FRA_4_c3</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_4 -- cost class 3</t>
   </si>
   <si>
-    <t>e_won-FRA_4_c2</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_4 -- cost class 2</t>
-  </si>
-  <si>
     <t>e_won-FRA_4_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_4 -- cost class 1</t>
   </si>
   <si>
+    <t>e_won-FRA_4_c5</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_4 -- cost class 5</t>
+  </si>
+  <si>
     <t>e_won-FRA_4_c4</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_4 -- cost class 4</t>
   </si>
   <si>
-    <t>e_won-FRA_4_c5</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_4 -- cost class 5</t>
+    <t>e_won-FRA_3_c1</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_3 -- cost class 1</t>
   </si>
   <si>
     <t>e_won-FRA_3_c2</t>
@@ -2362,40 +2368,34 @@
     <t>onshore wind resource -- CF class won-FRA_3 -- cost class 2</t>
   </si>
   <si>
-    <t>e_won-FRA_3_c1</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_3 -- cost class 1</t>
-  </si>
-  <si>
     <t>e_won-FRA_2_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_2 -- cost class 1</t>
   </si>
   <si>
+    <t>e_won-FRA_2_c3</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_2 -- cost class 3</t>
+  </si>
+  <si>
     <t>e_won-FRA_2_c2</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_2 -- cost class 2</t>
   </si>
   <si>
-    <t>e_won-FRA_2_c3</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_2 -- cost class 3</t>
+    <t>e_won-FRA_2_c4</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-FRA_2 -- cost class 4</t>
   </si>
   <si>
     <t>e_won-FRA_2_c5</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-FRA_2 -- cost class 5</t>
-  </si>
-  <si>
-    <t>e_won-FRA_2_c4</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-FRA_2 -- cost class 4</t>
   </si>
   <si>
     <t>e_won-FRA_1_c1</t>
@@ -8016,7 +8016,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7F57F98-29A8-46AB-B6CA-C2871539405A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F769103-B9CE-45E4-926E-7AC445CB52EE}">
   <dimension ref="B9:N55"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9782,7 +9782,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{472EE37A-E776-4035-9580-A4DE53FC1CEC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD93C00D-FE11-4FCA-A193-0C295B0816C2}">
   <dimension ref="B9:AB253"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9909,7 +9909,7 @@
         <v>0.60125972819957696</v>
       </c>
       <c r="N11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P11" t="s">
         <v>182</v>
@@ -9983,7 +9983,7 @@
         <v>0.60125972819957696</v>
       </c>
       <c r="N12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P12" t="s">
         <v>182</v>
@@ -10797,7 +10797,7 @@
         <v>0.57376405752186443</v>
       </c>
       <c r="N23">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P23" t="s">
         <v>182</v>
@@ -10871,7 +10871,7 @@
         <v>0.57376405752186443</v>
       </c>
       <c r="N24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P24" t="s">
         <v>182</v>
@@ -11019,7 +11019,7 @@
         <v>0.56435453053259388</v>
       </c>
       <c r="N26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P26" t="s">
         <v>182</v>
@@ -11093,7 +11093,7 @@
         <v>0.56435453053259388</v>
       </c>
       <c r="N27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P27" t="s">
         <v>182</v>
@@ -11167,7 +11167,7 @@
         <v>0.5481425465611397</v>
       </c>
       <c r="N28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P28" t="s">
         <v>182</v>
@@ -11241,7 +11241,7 @@
         <v>0.5481425465611397</v>
       </c>
       <c r="N29">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P29" t="s">
         <v>182</v>
@@ -11463,7 +11463,7 @@
         <v>0.53797007154491827</v>
       </c>
       <c r="N32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P32" t="s">
         <v>182</v>
@@ -11537,7 +11537,7 @@
         <v>0.53797007154491827</v>
       </c>
       <c r="N33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P33" t="s">
         <v>182</v>
@@ -11685,7 +11685,7 @@
         <v>0.53220597567372174</v>
       </c>
       <c r="N35">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P35" t="s">
         <v>182</v>
@@ -11759,7 +11759,7 @@
         <v>0.53220597567372174</v>
       </c>
       <c r="N36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P36" t="s">
         <v>182</v>
@@ -11981,7 +11981,7 @@
         <v>0.50220459612144741</v>
       </c>
       <c r="N39">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P39" t="s">
         <v>182</v>
@@ -12055,7 +12055,7 @@
         <v>0.50220459612144741</v>
       </c>
       <c r="N40">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P40" t="s">
         <v>182</v>
@@ -12129,7 +12129,7 @@
         <v>0.49522886431330682</v>
       </c>
       <c r="N41">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P41" t="s">
         <v>182</v>
@@ -12203,7 +12203,7 @@
         <v>0.49522886431330682</v>
       </c>
       <c r="N42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P42" t="s">
         <v>182</v>
@@ -12425,7 +12425,7 @@
         <v>0.48997678015376445</v>
       </c>
       <c r="N45">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P45" t="s">
         <v>182</v>
@@ -12499,7 +12499,7 @@
         <v>0.48997678015376445</v>
       </c>
       <c r="N46">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P46" t="s">
         <v>182</v>
@@ -12647,7 +12647,7 @@
         <v>0.48274206530326413</v>
       </c>
       <c r="N48">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P48" t="s">
         <v>182</v>
@@ -12721,7 +12721,7 @@
         <v>0.48274206530326413</v>
       </c>
       <c r="N49">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P49" t="s">
         <v>182</v>
@@ -12795,7 +12795,7 @@
         <v>0.47674972936727938</v>
       </c>
       <c r="N50">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P50" t="s">
         <v>182</v>
@@ -12869,7 +12869,7 @@
         <v>0.47674972936727938</v>
       </c>
       <c r="N51">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P51" t="s">
         <v>182</v>
@@ -13313,7 +13313,7 @@
         <v>0.46248796199573244</v>
       </c>
       <c r="N57">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P57" t="s">
         <v>182</v>
@@ -13387,7 +13387,7 @@
         <v>0.46248796199573244</v>
       </c>
       <c r="N58">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P58" t="s">
         <v>182</v>
@@ -13461,7 +13461,7 @@
         <v>0.45706678449843924</v>
       </c>
       <c r="N59">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P59" t="s">
         <v>182</v>
@@ -13535,7 +13535,7 @@
         <v>0.45706678449843924</v>
       </c>
       <c r="N60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P60" t="s">
         <v>182</v>
@@ -13609,7 +13609,7 @@
         <v>0.45017606551383099</v>
       </c>
       <c r="N61">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P61" t="s">
         <v>182</v>
@@ -13683,7 +13683,7 @@
         <v>0.45017606551383099</v>
       </c>
       <c r="N62">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P62" t="s">
         <v>182</v>
@@ -13757,7 +13757,7 @@
         <v>0.44927182040159591</v>
       </c>
       <c r="N63">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P63" t="s">
         <v>182</v>
@@ -13831,7 +13831,7 @@
         <v>0.44927182040159591</v>
       </c>
       <c r="N64">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P64" t="s">
         <v>182</v>
@@ -13905,7 +13905,7 @@
         <v>0.4311669102324972</v>
       </c>
       <c r="N65">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P65" t="s">
         <v>182</v>
@@ -13979,7 +13979,7 @@
         <v>0.4311669102324972</v>
       </c>
       <c r="N66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P66" t="s">
         <v>182</v>
@@ -14053,7 +14053,7 @@
         <v>0.42909230521710767</v>
       </c>
       <c r="N67">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P67" t="s">
         <v>182</v>
@@ -14127,7 +14127,7 @@
         <v>0.42909230521710767</v>
       </c>
       <c r="N68">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P68" t="s">
         <v>182</v>
@@ -14201,7 +14201,7 @@
         <v>0.42022316971090101</v>
       </c>
       <c r="N69">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P69" t="s">
         <v>182</v>
@@ -14275,7 +14275,7 @@
         <v>0.42022316971090101</v>
       </c>
       <c r="N70">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P70" t="s">
         <v>182</v>
@@ -14423,7 +14423,7 @@
         <v>0.41247392735747213</v>
       </c>
       <c r="N72">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P72" t="s">
         <v>182</v>
@@ -14497,7 +14497,7 @@
         <v>0.41247392735747213</v>
       </c>
       <c r="N73">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P73" t="s">
         <v>182</v>
@@ -14719,7 +14719,7 @@
         <v>0.40413001707392909</v>
       </c>
       <c r="N76">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P76" t="s">
         <v>182</v>
@@ -14793,7 +14793,7 @@
         <v>0.40413001707392909</v>
       </c>
       <c r="N77">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P77" t="s">
         <v>182</v>
@@ -14941,7 +14941,7 @@
         <v>0.3980373835402759</v>
       </c>
       <c r="N79">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P79" t="s">
         <v>182</v>
@@ -15015,7 +15015,7 @@
         <v>0.3980373835402759</v>
       </c>
       <c r="N80">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P80" t="s">
         <v>182</v>
@@ -15237,7 +15237,7 @@
         <v>0.38888490739692388</v>
       </c>
       <c r="N83">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P83" t="s">
         <v>182</v>
@@ -15311,7 +15311,7 @@
         <v>0.38888490739692388</v>
       </c>
       <c r="N84">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P84" t="s">
         <v>182</v>
@@ -20789,7 +20789,7 @@
         <v>0.14818841965104529</v>
       </c>
       <c r="N195">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="196" spans="2:14">
@@ -20827,7 +20827,7 @@
         <v>0.14818841965104529</v>
       </c>
       <c r="N196">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="197" spans="2:14">
@@ -20903,7 +20903,7 @@
         <v>0.13893757467141449</v>
       </c>
       <c r="N198">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="199" spans="2:14">
@@ -20941,7 +20941,7 @@
         <v>0.13893757467141449</v>
       </c>
       <c r="N199">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="200" spans="2:14">
@@ -21055,7 +21055,7 @@
         <v>0.13455537949825541</v>
       </c>
       <c r="N202">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="203" spans="2:14">
@@ -21093,7 +21093,7 @@
         <v>0.13455537949825541</v>
       </c>
       <c r="N203">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="204" spans="2:14">
@@ -21321,7 +21321,7 @@
         <v>0.1136420932326222</v>
       </c>
       <c r="N209">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="210" spans="2:14">
@@ -21359,7 +21359,7 @@
         <v>0.1136420932326222</v>
       </c>
       <c r="N210">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="211" spans="2:14">
@@ -21511,7 +21511,7 @@
         <v>9.7592962323386184E-2</v>
       </c>
       <c r="N214">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="215" spans="2:14">
@@ -21549,7 +21549,7 @@
         <v>9.7592962323386184E-2</v>
       </c>
       <c r="N215">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="216" spans="2:14">
@@ -21587,7 +21587,7 @@
         <v>9.6601232604683201E-2</v>
       </c>
       <c r="N216">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="217" spans="2:14">
@@ -21625,7 +21625,7 @@
         <v>9.6601232604683201E-2</v>
       </c>
       <c r="N217">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="218" spans="2:14">
@@ -21815,7 +21815,7 @@
         <v>8.3146820266911795E-2</v>
       </c>
       <c r="N222">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="223" spans="2:14">
@@ -21853,7 +21853,7 @@
         <v>8.3146820266911795E-2</v>
       </c>
       <c r="N223">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="224" spans="2:14">
@@ -22385,7 +22385,7 @@
         <v>4.4893033534251302E-2</v>
       </c>
       <c r="N237">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="238" spans="2:14">
@@ -22423,7 +22423,7 @@
         <v>4.4893033534251302E-2</v>
       </c>
       <c r="N238">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="239" spans="2:14">
@@ -22499,7 +22499,7 @@
         <v>3.6383893461016302E-2</v>
       </c>
       <c r="N240">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="241" spans="2:14">
@@ -22537,7 +22537,7 @@
         <v>3.6383893461016302E-2</v>
       </c>
       <c r="N241">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="242" spans="2:14">
@@ -22575,7 +22575,7 @@
         <v>2.6841442574643999E-2</v>
       </c>
       <c r="N242">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="243" spans="2:14">
@@ -22613,7 +22613,7 @@
         <v>2.6841442574643999E-2</v>
       </c>
       <c r="N243">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="244" spans="2:14">
@@ -22689,7 +22689,7 @@
         <v>1.7038190092558199E-2</v>
       </c>
       <c r="N245">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="246" spans="2:14">
@@ -22727,7 +22727,7 @@
         <v>1.7038190092558199E-2</v>
       </c>
       <c r="N246">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="247" spans="2:14">
@@ -22765,7 +22765,7 @@
         <v>1.58504479105879E-2</v>
       </c>
       <c r="N247">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="248" spans="2:14">
@@ -22803,7 +22803,7 @@
         <v>1.58504479105879E-2</v>
       </c>
       <c r="N248">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="249" spans="2:14">
@@ -23002,7 +23002,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE099407-1872-420B-998F-B75BBFE06647}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA3440AE-C36F-4E8E-9E04-52A7E7645AEB}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>